<commit_message>
feat(registry): close final 13 IAST manually (600/600 verified); add D1 registry system — schema.sql (entities/entity_names/entity_categories/entity_relations), idempotent registry_load.py loader, registry-load GitHub Actions workflow
</commit_message>
<xml_diff>
--- a/docs/entity-registry/ISKCON_Glossary.xlsx
+++ b/docs/entity-registry/ISKCON_Glossary.xlsx
@@ -2661,12 +2661,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Brihachchishu</t>
+          <t>Bṛhacchiṣu</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -8133,12 +8133,12 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Vīrā-Devī I Dūtī-Devī</t>
+          <t>Vīrā-devī / Dūtī-devī</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr"/>
@@ -12931,12 +12931,12 @@
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>Jānakī I Rukmiṇī</t>
+          <t>Jānakī / Rukmiṇī</t>
         </is>
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr"/>
@@ -13049,12 +13049,12 @@
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>Jangali</t>
+          <t>Jāṅgalī</t>
         </is>
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -16064,12 +16064,12 @@
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t>Kārttikeya I Acyuta-Gopī</t>
+          <t>Kārttikeya / Acyuta-gopī</t>
         </is>
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -18115,12 +18115,12 @@
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>Lavanga/rati-Mañjarī I Sanātana Kumāra</t>
+          <t>Lavaṅga-mañjarī / Rati-mañjarī</t>
         </is>
       </c>
       <c r="F299" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G299" s="2" t="inlineStr">
@@ -21858,12 +21858,12 @@
       </c>
       <c r="E362" s="2" t="inlineStr">
         <is>
-          <t>Nanday</t>
+          <t>Nandāi</t>
         </is>
       </c>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G362" s="2" t="inlineStr">
@@ -26505,12 +26505,12 @@
       </c>
       <c r="E441" s="2" t="inlineStr">
         <is>
-          <t>Ramay</t>
+          <t>Rāmāi</t>
         </is>
       </c>
       <c r="F441" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G441" s="2" t="inlineStr">
@@ -27030,12 +27030,12 @@
       </c>
       <c r="E450" s="2" t="inlineStr">
         <is>
-          <t>Rasa/rati-Mañjarī</t>
+          <t>Rāsa-mañjarī / Rati-mañjarī</t>
         </is>
       </c>
       <c r="F450" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G450" s="2" t="inlineStr">
@@ -31713,12 +31713,12 @@
       </c>
       <c r="E529" s="2" t="inlineStr">
         <is>
-          <t>Phleyta Gospoda Krishny</t>
+          <t>Vaṁśī</t>
         </is>
       </c>
       <c r="F529" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G529" s="2" t="inlineStr"/>
@@ -33198,12 +33198,12 @@
       </c>
       <c r="E554" s="2" t="inlineStr">
         <is>
-          <t>Candrakānti-Devī I Pūrṇānanda-Gopī</t>
+          <t>Candrakānti-devī / Pūrṇānanda-gopī</t>
         </is>
       </c>
       <c r="F554" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G554" s="2" t="inlineStr">
@@ -33792,12 +33792,12 @@
       </c>
       <c r="E564" s="2" t="inlineStr">
         <is>
-          <t>Śaibyā-Gopī I Sarasvatī</t>
+          <t>Śaibyā-gopī / Sarasvatī</t>
         </is>
       </c>
       <c r="F564" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G564" s="2" t="inlineStr">
@@ -35733,12 +35733,12 @@
       </c>
       <c r="E597" s="2" t="inlineStr">
         <is>
-          <t>Yagya-Patnī</t>
+          <t>Yajña-patnī</t>
         </is>
       </c>
       <c r="F597" s="2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="G597" s="2" t="inlineStr"/>

</xml_diff>